<commit_message>
Update MM scripts, notebooks, and outputs
</commit_message>
<xml_diff>
--- a/2025_bracket_preds.xlsx
+++ b/2025_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>98.59999999999999</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>71.8</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>50.8</v>
+        <v>54</v>
       </c>
       <c r="J2" t="n">
-        <v>34.1</v>
+        <v>36.1</v>
       </c>
       <c r="K2" t="n">
-        <v>20.5</v>
+        <v>22.4</v>
       </c>
       <c r="L2" t="n">
-        <v>11.3</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="3">
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>80.7</v>
+        <v>80.2</v>
       </c>
       <c r="H3" t="n">
-        <v>56.5</v>
+        <v>55</v>
       </c>
       <c r="I3" t="n">
-        <v>37</v>
+        <v>33.5</v>
       </c>
       <c r="J3" t="n">
-        <v>21.1</v>
+        <v>18.4</v>
       </c>
       <c r="K3" t="n">
-        <v>12.1</v>
+        <v>10.5</v>
       </c>
       <c r="L3" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="4">
@@ -592,22 +592,22 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>93.09999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="H4" t="n">
-        <v>55.5</v>
+        <v>55.8</v>
       </c>
       <c r="I4" t="n">
-        <v>26.6</v>
+        <v>29.4</v>
       </c>
       <c r="J4" t="n">
-        <v>10.9</v>
+        <v>12.6</v>
       </c>
       <c r="K4" t="n">
-        <v>5.1</v>
+        <v>5.8</v>
       </c>
       <c r="L4" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="5">
@@ -636,22 +636,22 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>81</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>54.1</v>
+        <v>50.9</v>
       </c>
       <c r="I5" t="n">
-        <v>22.2</v>
+        <v>18.8</v>
       </c>
       <c r="J5" t="n">
-        <v>10.5</v>
+        <v>8.9</v>
       </c>
       <c r="K5" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="L5" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6">
@@ -680,22 +680,22 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>27.4</v>
+        <v>34.2</v>
       </c>
       <c r="I6" t="n">
-        <v>9.1</v>
+        <v>11</v>
       </c>
       <c r="J6" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="K6" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7">
@@ -724,22 +724,22 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>56.1</v>
+        <v>56</v>
       </c>
       <c r="H7" t="n">
-        <v>26.7</v>
+        <v>26.2</v>
       </c>
       <c r="I7" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="J7" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="K7" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
@@ -768,22 +768,22 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>68.3</v>
+        <v>65.7</v>
       </c>
       <c r="H8" t="n">
-        <v>29.3</v>
+        <v>29.8</v>
       </c>
       <c r="I8" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="J8" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="K8" t="n">
         <v>1.8</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="9">
@@ -812,19 +812,19 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>51.3</v>
+        <v>47.2</v>
       </c>
       <c r="H9" t="n">
-        <v>15.3</v>
+        <v>12.6</v>
       </c>
       <c r="I9" t="n">
-        <v>7.7</v>
+        <v>6.5</v>
       </c>
       <c r="J9" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="K9" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="L9" t="n">
         <v>0.3</v>
@@ -856,22 +856,22 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>48.7</v>
+        <v>52.8</v>
       </c>
       <c r="H10" t="n">
-        <v>12.9</v>
+        <v>14.1</v>
       </c>
       <c r="I10" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="J10" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="K10" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="11">
@@ -900,13 +900,13 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>31.6</v>
+        <v>34.3</v>
       </c>
       <c r="H11" t="n">
-        <v>10.8</v>
+        <v>12.4</v>
       </c>
       <c r="I11" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -944,22 +944,22 @@
         <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>43.9</v>
+        <v>44</v>
       </c>
       <c r="H12" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="I12" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="J12" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="K12" t="n">
         <v>0.9</v>
       </c>
       <c r="L12" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="13">
@@ -988,22 +988,22 @@
         <v>100</v>
       </c>
       <c r="G13" t="n">
-        <v>37.1</v>
+        <v>29.1</v>
       </c>
       <c r="H13" t="n">
-        <v>13.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>2.7</v>
+        <v>1.8</v>
       </c>
       <c r="J13" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1032,10 +1032,10 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="H14" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="I14" t="n">
         <v>0.7</v>
@@ -1076,7 +1076,7 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>6.9</v>
+        <v>7.6</v>
       </c>
       <c r="H15" t="n">
         <v>0.7</v>
@@ -1120,13 +1120,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>19.3</v>
+        <v>19.8</v>
       </c>
       <c r="H16" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J16" t="n">
         <v>0.1</v>
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>47.6</v>
+        <v>46.1</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -1205,10 +1205,10 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>52.4</v>
+        <v>53.9</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="H18" t="n">
         <v>0.1</v>
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>99</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>72.5</v>
+        <v>67.7</v>
       </c>
       <c r="I19" t="n">
-        <v>52.5</v>
+        <v>48.9</v>
       </c>
       <c r="J19" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="K19" t="n">
-        <v>19.1</v>
+        <v>17.7</v>
       </c>
       <c r="L19" t="n">
-        <v>10.7</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1296,22 +1296,22 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>85.7</v>
+        <v>88</v>
       </c>
       <c r="H20" t="n">
-        <v>60.8</v>
+        <v>63.6</v>
       </c>
       <c r="I20" t="n">
-        <v>41.5</v>
+        <v>42.8</v>
       </c>
       <c r="J20" t="n">
-        <v>24.2</v>
+        <v>25.3</v>
       </c>
       <c r="K20" t="n">
-        <v>13.4</v>
+        <v>14.1</v>
       </c>
       <c r="L20" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1340,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H21" t="n">
-        <v>39.3</v>
+        <v>38.5</v>
       </c>
       <c r="I21" t="n">
-        <v>17.1</v>
+        <v>16.8</v>
       </c>
       <c r="J21" t="n">
         <v>7.3</v>
       </c>
       <c r="K21" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1384,19 +1384,19 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>72.3</v>
+        <v>72.7</v>
       </c>
       <c r="H22" t="n">
-        <v>43.6</v>
+        <v>44.1</v>
       </c>
       <c r="I22" t="n">
-        <v>16.4</v>
+        <v>18.1</v>
       </c>
       <c r="J22" t="n">
-        <v>7.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="L22" t="n">
         <v>1.1</v>
@@ -1428,19 +1428,19 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>76.3</v>
+        <v>76.5</v>
       </c>
       <c r="H23" t="n">
-        <v>39.9</v>
+        <v>39.8</v>
       </c>
       <c r="I23" t="n">
-        <v>12.9</v>
+        <v>12.6</v>
       </c>
       <c r="J23" t="n">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="K23" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="L23" t="n">
         <v>0.8</v>
@@ -1472,19 +1472,19 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>68.2</v>
+        <v>66.5</v>
       </c>
       <c r="H24" t="n">
-        <v>37.9</v>
+        <v>38.7</v>
       </c>
       <c r="I24" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
       <c r="J24" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="K24" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -1516,22 +1516,22 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>63.7</v>
+        <v>55.8</v>
       </c>
       <c r="H25" t="n">
-        <v>23.2</v>
+        <v>18.9</v>
       </c>
       <c r="I25" t="n">
-        <v>11.2</v>
+        <v>9.4</v>
       </c>
       <c r="J25" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="K25" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="26">
@@ -1563,19 +1563,19 @@
         <v>63.7</v>
       </c>
       <c r="H26" t="n">
-        <v>20.4</v>
+        <v>22.6</v>
       </c>
       <c r="I26" t="n">
-        <v>12.1</v>
+        <v>13.3</v>
       </c>
       <c r="J26" t="n">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="K26" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="27">
@@ -1607,16 +1607,16 @@
         <v>36.3</v>
       </c>
       <c r="H27" t="n">
-        <v>7.1</v>
+        <v>9.5</v>
       </c>
       <c r="I27" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="J27" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="K27" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L27" t="n">
         <v>0.2</v>
@@ -1648,22 +1648,22 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>36.3</v>
+        <v>44.2</v>
       </c>
       <c r="H28" t="n">
-        <v>13.3</v>
+        <v>15.3</v>
       </c>
       <c r="I28" t="n">
-        <v>5.2</v>
+        <v>6.5</v>
       </c>
       <c r="J28" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="K28" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L28" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="29">
@@ -1689,16 +1689,16 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>52.4</v>
+        <v>53.6</v>
       </c>
       <c r="G29" t="n">
-        <v>16.8</v>
+        <v>18.6</v>
       </c>
       <c r="H29" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I29" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -1733,19 +1733,19 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>47.6</v>
+        <v>46.4</v>
       </c>
       <c r="G30" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="H30" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="I30" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="J30" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="K30" t="n">
         <v>0.1</v>
@@ -1780,16 +1780,16 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>23.7</v>
+        <v>23.5</v>
       </c>
       <c r="H31" t="n">
         <v>8.5</v>
       </c>
       <c r="I31" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="J31" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K31" t="n">
         <v>0.1</v>
@@ -1824,10 +1824,10 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>27.7</v>
+        <v>27.3</v>
       </c>
       <c r="H32" t="n">
-        <v>8</v>
+        <v>7.6</v>
       </c>
       <c r="I32" t="n">
         <v>1.1</v>
@@ -1836,7 +1836,7 @@
         <v>0.3</v>
       </c>
       <c r="K32" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -1868,16 +1868,16 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H33" t="n">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I33" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="J33" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K33" t="n">
         <v>0.1</v>
@@ -1912,16 +1912,16 @@
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>14.3</v>
+        <v>12</v>
       </c>
       <c r="H34" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="I34" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1956,10 +1956,10 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>3.9</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2000,16 +2000,16 @@
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>97.3</v>
+        <v>96.7</v>
       </c>
       <c r="H36" t="n">
-        <v>74.7</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="I36" t="n">
-        <v>56.2</v>
+        <v>56.7</v>
       </c>
       <c r="J36" t="n">
-        <v>39.2</v>
+        <v>39</v>
       </c>
       <c r="K36" t="n">
         <v>25.3</v>
@@ -2044,22 +2044,22 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>91</v>
+        <v>92.5</v>
       </c>
       <c r="H37" t="n">
-        <v>60.1</v>
+        <v>61.7</v>
       </c>
       <c r="I37" t="n">
         <v>38.5</v>
       </c>
       <c r="J37" t="n">
-        <v>17.9</v>
+        <v>18.9</v>
       </c>
       <c r="K37" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="L37" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="38">
@@ -2088,22 +2088,22 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>80.5</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>55</v>
+        <v>54.6</v>
       </c>
       <c r="I38" t="n">
-        <v>27.7</v>
+        <v>28.2</v>
       </c>
       <c r="J38" t="n">
-        <v>12.7</v>
+        <v>13.3</v>
       </c>
       <c r="K38" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="L38" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="39">
@@ -2132,22 +2132,22 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>76.90000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>44.5</v>
+        <v>40.6</v>
       </c>
       <c r="I39" t="n">
-        <v>15.3</v>
+        <v>13.2</v>
       </c>
       <c r="J39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K39" t="n">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
       <c r="L39" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="40">
@@ -2176,19 +2176,19 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>60</v>
+        <v>54.9</v>
       </c>
       <c r="H40" t="n">
-        <v>31.1</v>
+        <v>28.6</v>
       </c>
       <c r="I40" t="n">
-        <v>9.699999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J40" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="K40" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="L40" t="n">
         <v>0.5</v>
@@ -2220,22 +2220,22 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>53.8</v>
+        <v>54.3</v>
       </c>
       <c r="H41" t="n">
-        <v>22.3</v>
+        <v>23.1</v>
       </c>
       <c r="I41" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J41" t="n">
         <v>3.1</v>
       </c>
       <c r="K41" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L41" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="42">
@@ -2264,22 +2264,22 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>63.8</v>
+        <v>65.8</v>
       </c>
       <c r="H42" t="n">
-        <v>26.4</v>
+        <v>26.7</v>
       </c>
       <c r="I42" t="n">
         <v>13.8</v>
       </c>
       <c r="J42" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="K42" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="L42" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="43">
@@ -2308,16 +2308,16 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>55.8</v>
+        <v>59</v>
       </c>
       <c r="H43" t="n">
-        <v>13.7</v>
+        <v>14.6</v>
       </c>
       <c r="I43" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="J43" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="K43" t="n">
         <v>1</v>
@@ -2352,19 +2352,19 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>44.2</v>
+        <v>41</v>
       </c>
       <c r="H44" t="n">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="I44" t="n">
-        <v>5.5</v>
+        <v>4.7</v>
       </c>
       <c r="J44" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K44" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L44" t="n">
         <v>0.1</v>
@@ -2396,19 +2396,19 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>36.2</v>
+        <v>34.2</v>
       </c>
       <c r="H45" t="n">
-        <v>11.9</v>
+        <v>10.6</v>
       </c>
       <c r="I45" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="J45" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K45" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L45" t="n">
         <v>0.1</v>
@@ -2437,19 +2437,19 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>55.5</v>
+        <v>55.4</v>
       </c>
       <c r="G46" t="n">
-        <v>26.3</v>
+        <v>25.7</v>
       </c>
       <c r="H46" t="n">
-        <v>11.1</v>
+        <v>10.6</v>
       </c>
       <c r="I46" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="J46" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="K46" t="n">
         <v>0.4</v>
@@ -2481,22 +2481,22 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>44.5</v>
+        <v>44.6</v>
       </c>
       <c r="G47" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="H47" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="I47" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="J47" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="K47" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L47" t="n">
         <v>0</v>
@@ -2528,19 +2528,19 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>40</v>
+        <v>45.1</v>
       </c>
       <c r="H48" t="n">
-        <v>17.1</v>
+        <v>22.4</v>
       </c>
       <c r="I48" t="n">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="J48" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="K48" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="L48" t="n">
         <v>0.1</v>
@@ -2572,22 +2572,22 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>23.1</v>
+        <v>25.4</v>
       </c>
       <c r="H49" t="n">
-        <v>7.4</v>
+        <v>8.4</v>
       </c>
       <c r="I49" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="J49" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K49" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L49" t="n">
         <v>0.1</v>
-      </c>
-      <c r="L49" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -2616,10 +2616,10 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>19.5</v>
+        <v>19.1</v>
       </c>
       <c r="H50" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="I50" t="n">
         <v>0.8</v>
@@ -2660,13 +2660,13 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2701,13 +2701,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>67.8</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="G52" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2745,13 +2745,13 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>32.2</v>
+        <v>34.9</v>
       </c>
       <c r="G53" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>94.5</v>
+        <v>95.5</v>
       </c>
       <c r="H54" t="n">
-        <v>75.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>57.7</v>
+        <v>60</v>
       </c>
       <c r="J54" t="n">
-        <v>41.9</v>
+        <v>44.8</v>
       </c>
       <c r="K54" t="n">
-        <v>26.5</v>
+        <v>27.8</v>
       </c>
       <c r="L54" t="n">
-        <v>16.4</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="55">
@@ -2836,19 +2836,19 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>93.59999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="H55" t="n">
-        <v>58.4</v>
+        <v>57.6</v>
       </c>
       <c r="I55" t="n">
-        <v>30.2</v>
+        <v>31.1</v>
       </c>
       <c r="J55" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="K55" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="L55" t="n">
         <v>2.5</v>
@@ -2880,22 +2880,22 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>80.5</v>
+        <v>76.8</v>
       </c>
       <c r="H56" t="n">
-        <v>51.3</v>
+        <v>48.4</v>
       </c>
       <c r="I56" t="n">
-        <v>30.4</v>
+        <v>29</v>
       </c>
       <c r="J56" t="n">
-        <v>13.8</v>
+        <v>12.3</v>
       </c>
       <c r="K56" t="n">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="L56" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="57">
@@ -2924,22 +2924,22 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>80.90000000000001</v>
+        <v>81.2</v>
       </c>
       <c r="H57" t="n">
-        <v>55.6</v>
+        <v>56.8</v>
       </c>
       <c r="I57" t="n">
-        <v>19.5</v>
+        <v>18.4</v>
       </c>
       <c r="J57" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="K57" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="L57" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="58">
@@ -2968,19 +2968,19 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>56.7</v>
+        <v>57.4</v>
       </c>
       <c r="H58" t="n">
-        <v>24.7</v>
+        <v>24</v>
       </c>
       <c r="I58" t="n">
-        <v>7</v>
+        <v>6.3</v>
       </c>
       <c r="J58" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="K58" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L58" t="n">
         <v>0.2</v>
@@ -3012,19 +3012,19 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>59.2</v>
+        <v>64.3</v>
       </c>
       <c r="H59" t="n">
-        <v>28.2</v>
+        <v>31.6</v>
       </c>
       <c r="I59" t="n">
-        <v>14.3</v>
+        <v>16.3</v>
       </c>
       <c r="J59" t="n">
-        <v>4.6</v>
+        <v>5.2</v>
       </c>
       <c r="K59" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="L59" t="n">
         <v>0.5</v>
@@ -3056,19 +3056,19 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>63.6</v>
+        <v>64.3</v>
       </c>
       <c r="H60" t="n">
-        <v>28.3</v>
+        <v>29</v>
       </c>
       <c r="I60" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="J60" t="n">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
       <c r="K60" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="L60" t="n">
         <v>0.5</v>
@@ -3100,19 +3100,19 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>61.3</v>
+        <v>66.5</v>
       </c>
       <c r="H61" t="n">
-        <v>14.4</v>
+        <v>15.1</v>
       </c>
       <c r="I61" t="n">
-        <v>7.4</v>
+        <v>8.1</v>
       </c>
       <c r="J61" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="K61" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="L61" t="n">
         <v>0.5</v>
@@ -3144,22 +3144,22 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>38.7</v>
+        <v>33.5</v>
       </c>
       <c r="H62" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
       <c r="I62" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="J62" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K62" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="L62" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="63">
@@ -3188,22 +3188,22 @@
         <v>100</v>
       </c>
       <c r="G63" t="n">
-        <v>36.4</v>
+        <v>35.7</v>
       </c>
       <c r="H63" t="n">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
       <c r="I63" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="K63" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L63" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -3232,22 +3232,22 @@
         <v>100</v>
       </c>
       <c r="G64" t="n">
-        <v>40.8</v>
+        <v>35.7</v>
       </c>
       <c r="H64" t="n">
-        <v>16.4</v>
+        <v>14.2</v>
       </c>
       <c r="I64" t="n">
-        <v>6.7</v>
+        <v>5.5</v>
       </c>
       <c r="J64" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="K64" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="L64" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="65">
@@ -3276,16 +3276,16 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>43.3</v>
+        <v>42.6</v>
       </c>
       <c r="H65" t="n">
-        <v>14.4</v>
+        <v>13.9</v>
       </c>
       <c r="I65" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="J65" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="K65" t="n">
         <v>0.3</v>
@@ -3320,7 +3320,7 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>19.1</v>
+        <v>18.8</v>
       </c>
       <c r="H66" t="n">
         <v>5.3</v>
@@ -3332,7 +3332,7 @@
         <v>0.2</v>
       </c>
       <c r="K66" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -3364,16 +3364,16 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>19.5</v>
+        <v>23.2</v>
       </c>
       <c r="H67" t="n">
-        <v>4</v>
+        <v>5.8</v>
       </c>
       <c r="I67" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="J67" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3408,7 +3408,7 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
       <c r="H68" t="n">
         <v>1.1</v>
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="H69" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I69" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Sync local main changes (20260308_124837)
</commit_message>
<xml_diff>
--- a/2025_bracket_preds.xlsx
+++ b/2025_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>98.59999999999999</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>71.8</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>50.8</v>
+        <v>54</v>
       </c>
       <c r="J2" t="n">
-        <v>34.1</v>
+        <v>36.1</v>
       </c>
       <c r="K2" t="n">
-        <v>20.5</v>
+        <v>22.4</v>
       </c>
       <c r="L2" t="n">
-        <v>11.3</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="3">
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>80.7</v>
+        <v>80.2</v>
       </c>
       <c r="H3" t="n">
-        <v>56.5</v>
+        <v>55</v>
       </c>
       <c r="I3" t="n">
-        <v>37</v>
+        <v>33.5</v>
       </c>
       <c r="J3" t="n">
-        <v>21.1</v>
+        <v>18.4</v>
       </c>
       <c r="K3" t="n">
-        <v>12.1</v>
+        <v>10.5</v>
       </c>
       <c r="L3" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="4">
@@ -592,22 +592,22 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>93.09999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="H4" t="n">
-        <v>55.5</v>
+        <v>55.8</v>
       </c>
       <c r="I4" t="n">
-        <v>26.6</v>
+        <v>29.4</v>
       </c>
       <c r="J4" t="n">
-        <v>10.9</v>
+        <v>12.6</v>
       </c>
       <c r="K4" t="n">
-        <v>5.1</v>
+        <v>5.8</v>
       </c>
       <c r="L4" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="5">
@@ -636,22 +636,22 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>81</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>54.1</v>
+        <v>50.9</v>
       </c>
       <c r="I5" t="n">
-        <v>22.2</v>
+        <v>18.8</v>
       </c>
       <c r="J5" t="n">
-        <v>10.5</v>
+        <v>8.9</v>
       </c>
       <c r="K5" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="L5" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="6">
@@ -680,22 +680,22 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>62.9</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>27.4</v>
+        <v>34.2</v>
       </c>
       <c r="I6" t="n">
-        <v>9.1</v>
+        <v>11</v>
       </c>
       <c r="J6" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="K6" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7">
@@ -724,22 +724,22 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>56.1</v>
+        <v>56</v>
       </c>
       <c r="H7" t="n">
-        <v>26.7</v>
+        <v>26.2</v>
       </c>
       <c r="I7" t="n">
-        <v>11.7</v>
+        <v>11.5</v>
       </c>
       <c r="J7" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="K7" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
@@ -768,22 +768,22 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>68.3</v>
+        <v>65.7</v>
       </c>
       <c r="H8" t="n">
-        <v>29.3</v>
+        <v>29.8</v>
       </c>
       <c r="I8" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="J8" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="K8" t="n">
         <v>1.8</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="9">
@@ -812,19 +812,19 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>51.3</v>
+        <v>47.2</v>
       </c>
       <c r="H9" t="n">
-        <v>15.3</v>
+        <v>12.6</v>
       </c>
       <c r="I9" t="n">
-        <v>7.7</v>
+        <v>6.5</v>
       </c>
       <c r="J9" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="K9" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="L9" t="n">
         <v>0.3</v>
@@ -856,22 +856,22 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>48.7</v>
+        <v>52.8</v>
       </c>
       <c r="H10" t="n">
-        <v>12.9</v>
+        <v>14.1</v>
       </c>
       <c r="I10" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="J10" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="K10" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="11">
@@ -900,13 +900,13 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>31.6</v>
+        <v>34.3</v>
       </c>
       <c r="H11" t="n">
-        <v>10.8</v>
+        <v>12.4</v>
       </c>
       <c r="I11" t="n">
-        <v>3.5</v>
+        <v>4.1</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -944,22 +944,22 @@
         <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>43.9</v>
+        <v>44</v>
       </c>
       <c r="H12" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="I12" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="J12" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="K12" t="n">
         <v>0.9</v>
       </c>
       <c r="L12" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="13">
@@ -988,22 +988,22 @@
         <v>100</v>
       </c>
       <c r="G13" t="n">
-        <v>37.1</v>
+        <v>29.1</v>
       </c>
       <c r="H13" t="n">
-        <v>13.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>2.7</v>
+        <v>1.8</v>
       </c>
       <c r="J13" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1032,10 +1032,10 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>19</v>
+        <v>18.9</v>
       </c>
       <c r="H14" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="I14" t="n">
         <v>0.7</v>
@@ -1076,7 +1076,7 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>6.9</v>
+        <v>7.6</v>
       </c>
       <c r="H15" t="n">
         <v>0.7</v>
@@ -1120,13 +1120,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>19.3</v>
+        <v>19.8</v>
       </c>
       <c r="H16" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J16" t="n">
         <v>0.1</v>
@@ -1161,13 +1161,13 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>47.6</v>
+        <v>46.1</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -1205,10 +1205,10 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>52.4</v>
+        <v>53.9</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="H18" t="n">
         <v>0.1</v>
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>99</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>72.5</v>
+        <v>67.7</v>
       </c>
       <c r="I19" t="n">
-        <v>52.5</v>
+        <v>48.9</v>
       </c>
       <c r="J19" t="n">
-        <v>32.5</v>
+        <v>30</v>
       </c>
       <c r="K19" t="n">
-        <v>19.1</v>
+        <v>17.7</v>
       </c>
       <c r="L19" t="n">
-        <v>10.7</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1296,22 +1296,22 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>85.7</v>
+        <v>88</v>
       </c>
       <c r="H20" t="n">
-        <v>60.8</v>
+        <v>63.6</v>
       </c>
       <c r="I20" t="n">
-        <v>41.5</v>
+        <v>42.8</v>
       </c>
       <c r="J20" t="n">
-        <v>24.2</v>
+        <v>25.3</v>
       </c>
       <c r="K20" t="n">
-        <v>13.4</v>
+        <v>14.1</v>
       </c>
       <c r="L20" t="n">
-        <v>7</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1340,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H21" t="n">
-        <v>39.3</v>
+        <v>38.5</v>
       </c>
       <c r="I21" t="n">
-        <v>17.1</v>
+        <v>16.8</v>
       </c>
       <c r="J21" t="n">
         <v>7.3</v>
       </c>
       <c r="K21" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1384,19 +1384,19 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>72.3</v>
+        <v>72.7</v>
       </c>
       <c r="H22" t="n">
-        <v>43.6</v>
+        <v>44.1</v>
       </c>
       <c r="I22" t="n">
-        <v>16.4</v>
+        <v>18.1</v>
       </c>
       <c r="J22" t="n">
-        <v>7.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="L22" t="n">
         <v>1.1</v>
@@ -1428,19 +1428,19 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>76.3</v>
+        <v>76.5</v>
       </c>
       <c r="H23" t="n">
-        <v>39.9</v>
+        <v>39.8</v>
       </c>
       <c r="I23" t="n">
-        <v>12.9</v>
+        <v>12.6</v>
       </c>
       <c r="J23" t="n">
-        <v>5.7</v>
+        <v>5.4</v>
       </c>
       <c r="K23" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="L23" t="n">
         <v>0.8</v>
@@ -1472,19 +1472,19 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>68.2</v>
+        <v>66.5</v>
       </c>
       <c r="H24" t="n">
-        <v>37.9</v>
+        <v>38.7</v>
       </c>
       <c r="I24" t="n">
-        <v>17.1</v>
+        <v>17.4</v>
       </c>
       <c r="J24" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
       <c r="K24" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
         <v>1</v>
@@ -1516,22 +1516,22 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>63.7</v>
+        <v>55.8</v>
       </c>
       <c r="H25" t="n">
-        <v>23.2</v>
+        <v>18.9</v>
       </c>
       <c r="I25" t="n">
-        <v>11.2</v>
+        <v>9.4</v>
       </c>
       <c r="J25" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="K25" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="26">
@@ -1563,19 +1563,19 @@
         <v>63.7</v>
       </c>
       <c r="H26" t="n">
-        <v>20.4</v>
+        <v>22.6</v>
       </c>
       <c r="I26" t="n">
-        <v>12.1</v>
+        <v>13.3</v>
       </c>
       <c r="J26" t="n">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="K26" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="L26" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="27">
@@ -1607,16 +1607,16 @@
         <v>36.3</v>
       </c>
       <c r="H27" t="n">
-        <v>7.1</v>
+        <v>9.5</v>
       </c>
       <c r="I27" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="J27" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="K27" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L27" t="n">
         <v>0.2</v>
@@ -1648,22 +1648,22 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>36.3</v>
+        <v>44.2</v>
       </c>
       <c r="H28" t="n">
-        <v>13.3</v>
+        <v>15.3</v>
       </c>
       <c r="I28" t="n">
-        <v>5.2</v>
+        <v>6.5</v>
       </c>
       <c r="J28" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="K28" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L28" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="29">
@@ -1689,16 +1689,16 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>52.4</v>
+        <v>53.6</v>
       </c>
       <c r="G29" t="n">
-        <v>16.8</v>
+        <v>18.6</v>
       </c>
       <c r="H29" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I29" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -1733,19 +1733,19 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>47.6</v>
+        <v>46.4</v>
       </c>
       <c r="G30" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="H30" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="I30" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="J30" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="K30" t="n">
         <v>0.1</v>
@@ -1780,16 +1780,16 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>23.7</v>
+        <v>23.5</v>
       </c>
       <c r="H31" t="n">
         <v>8.5</v>
       </c>
       <c r="I31" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="J31" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K31" t="n">
         <v>0.1</v>
@@ -1824,10 +1824,10 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>27.7</v>
+        <v>27.3</v>
       </c>
       <c r="H32" t="n">
-        <v>8</v>
+        <v>7.6</v>
       </c>
       <c r="I32" t="n">
         <v>1.1</v>
@@ -1836,7 +1836,7 @@
         <v>0.3</v>
       </c>
       <c r="K32" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -1868,16 +1868,16 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H33" t="n">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="I33" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="J33" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K33" t="n">
         <v>0.1</v>
@@ -1912,16 +1912,16 @@
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>14.3</v>
+        <v>12</v>
       </c>
       <c r="H34" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="I34" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1956,10 +1956,10 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>3.9</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2000,16 +2000,16 @@
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>97.3</v>
+        <v>96.7</v>
       </c>
       <c r="H36" t="n">
-        <v>74.7</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="I36" t="n">
-        <v>56.2</v>
+        <v>56.7</v>
       </c>
       <c r="J36" t="n">
-        <v>39.2</v>
+        <v>39</v>
       </c>
       <c r="K36" t="n">
         <v>25.3</v>
@@ -2044,22 +2044,22 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>91</v>
+        <v>92.5</v>
       </c>
       <c r="H37" t="n">
-        <v>60.1</v>
+        <v>61.7</v>
       </c>
       <c r="I37" t="n">
         <v>38.5</v>
       </c>
       <c r="J37" t="n">
-        <v>17.9</v>
+        <v>18.9</v>
       </c>
       <c r="K37" t="n">
-        <v>8.6</v>
+        <v>9.1</v>
       </c>
       <c r="L37" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="38">
@@ -2088,22 +2088,22 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>80.5</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>55</v>
+        <v>54.6</v>
       </c>
       <c r="I38" t="n">
-        <v>27.7</v>
+        <v>28.2</v>
       </c>
       <c r="J38" t="n">
-        <v>12.7</v>
+        <v>13.3</v>
       </c>
       <c r="K38" t="n">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="L38" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="39">
@@ -2132,22 +2132,22 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>76.90000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>44.5</v>
+        <v>40.6</v>
       </c>
       <c r="I39" t="n">
-        <v>15.3</v>
+        <v>13.2</v>
       </c>
       <c r="J39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K39" t="n">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
       <c r="L39" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="40">
@@ -2176,19 +2176,19 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>60</v>
+        <v>54.9</v>
       </c>
       <c r="H40" t="n">
-        <v>31.1</v>
+        <v>28.6</v>
       </c>
       <c r="I40" t="n">
-        <v>9.699999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J40" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="K40" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="L40" t="n">
         <v>0.5</v>
@@ -2220,22 +2220,22 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>53.8</v>
+        <v>54.3</v>
       </c>
       <c r="H41" t="n">
-        <v>22.3</v>
+        <v>23.1</v>
       </c>
       <c r="I41" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J41" t="n">
         <v>3.1</v>
       </c>
       <c r="K41" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L41" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="42">
@@ -2264,22 +2264,22 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>63.8</v>
+        <v>65.8</v>
       </c>
       <c r="H42" t="n">
-        <v>26.4</v>
+        <v>26.7</v>
       </c>
       <c r="I42" t="n">
         <v>13.8</v>
       </c>
       <c r="J42" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="K42" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="L42" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="43">
@@ -2308,16 +2308,16 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>55.8</v>
+        <v>59</v>
       </c>
       <c r="H43" t="n">
-        <v>13.7</v>
+        <v>14.6</v>
       </c>
       <c r="I43" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="J43" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="K43" t="n">
         <v>1</v>
@@ -2352,19 +2352,19 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>44.2</v>
+        <v>41</v>
       </c>
       <c r="H44" t="n">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="I44" t="n">
-        <v>5.5</v>
+        <v>4.7</v>
       </c>
       <c r="J44" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K44" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L44" t="n">
         <v>0.1</v>
@@ -2396,19 +2396,19 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>36.2</v>
+        <v>34.2</v>
       </c>
       <c r="H45" t="n">
-        <v>11.9</v>
+        <v>10.6</v>
       </c>
       <c r="I45" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="J45" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K45" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L45" t="n">
         <v>0.1</v>
@@ -2437,19 +2437,19 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>55.5</v>
+        <v>55.4</v>
       </c>
       <c r="G46" t="n">
-        <v>26.3</v>
+        <v>25.7</v>
       </c>
       <c r="H46" t="n">
-        <v>11.1</v>
+        <v>10.6</v>
       </c>
       <c r="I46" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="J46" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="K46" t="n">
         <v>0.4</v>
@@ -2481,22 +2481,22 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>44.5</v>
+        <v>44.6</v>
       </c>
       <c r="G47" t="n">
-        <v>19.9</v>
+        <v>20</v>
       </c>
       <c r="H47" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="I47" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="J47" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="K47" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L47" t="n">
         <v>0</v>
@@ -2528,19 +2528,19 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>40</v>
+        <v>45.1</v>
       </c>
       <c r="H48" t="n">
-        <v>17.1</v>
+        <v>22.4</v>
       </c>
       <c r="I48" t="n">
-        <v>4.5</v>
+        <v>6.7</v>
       </c>
       <c r="J48" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="K48" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="L48" t="n">
         <v>0.1</v>
@@ -2572,22 +2572,22 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>23.1</v>
+        <v>25.4</v>
       </c>
       <c r="H49" t="n">
-        <v>7.4</v>
+        <v>8.4</v>
       </c>
       <c r="I49" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="J49" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K49" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L49" t="n">
         <v>0.1</v>
-      </c>
-      <c r="L49" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -2616,10 +2616,10 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>19.5</v>
+        <v>19.1</v>
       </c>
       <c r="H50" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="I50" t="n">
         <v>0.8</v>
@@ -2660,13 +2660,13 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2701,13 +2701,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>67.8</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="G52" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2745,13 +2745,13 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>32.2</v>
+        <v>34.9</v>
       </c>
       <c r="G53" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>94.5</v>
+        <v>95.5</v>
       </c>
       <c r="H54" t="n">
-        <v>75.90000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>57.7</v>
+        <v>60</v>
       </c>
       <c r="J54" t="n">
-        <v>41.9</v>
+        <v>44.8</v>
       </c>
       <c r="K54" t="n">
-        <v>26.5</v>
+        <v>27.8</v>
       </c>
       <c r="L54" t="n">
-        <v>16.4</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="55">
@@ -2836,19 +2836,19 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>93.59999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="H55" t="n">
-        <v>58.4</v>
+        <v>57.6</v>
       </c>
       <c r="I55" t="n">
-        <v>30.2</v>
+        <v>31.1</v>
       </c>
       <c r="J55" t="n">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
       <c r="K55" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="L55" t="n">
         <v>2.5</v>
@@ -2880,22 +2880,22 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>80.5</v>
+        <v>76.8</v>
       </c>
       <c r="H56" t="n">
-        <v>51.3</v>
+        <v>48.4</v>
       </c>
       <c r="I56" t="n">
-        <v>30.4</v>
+        <v>29</v>
       </c>
       <c r="J56" t="n">
-        <v>13.8</v>
+        <v>12.3</v>
       </c>
       <c r="K56" t="n">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="L56" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="57">
@@ -2924,22 +2924,22 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>80.90000000000001</v>
+        <v>81.2</v>
       </c>
       <c r="H57" t="n">
-        <v>55.6</v>
+        <v>56.8</v>
       </c>
       <c r="I57" t="n">
-        <v>19.5</v>
+        <v>18.4</v>
       </c>
       <c r="J57" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="K57" t="n">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="L57" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="58">
@@ -2968,19 +2968,19 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>56.7</v>
+        <v>57.4</v>
       </c>
       <c r="H58" t="n">
-        <v>24.7</v>
+        <v>24</v>
       </c>
       <c r="I58" t="n">
-        <v>7</v>
+        <v>6.3</v>
       </c>
       <c r="J58" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="K58" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L58" t="n">
         <v>0.2</v>
@@ -3012,19 +3012,19 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>59.2</v>
+        <v>64.3</v>
       </c>
       <c r="H59" t="n">
-        <v>28.2</v>
+        <v>31.6</v>
       </c>
       <c r="I59" t="n">
-        <v>14.3</v>
+        <v>16.3</v>
       </c>
       <c r="J59" t="n">
-        <v>4.6</v>
+        <v>5.2</v>
       </c>
       <c r="K59" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="L59" t="n">
         <v>0.5</v>
@@ -3056,19 +3056,19 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>63.6</v>
+        <v>64.3</v>
       </c>
       <c r="H60" t="n">
-        <v>28.3</v>
+        <v>29</v>
       </c>
       <c r="I60" t="n">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
       <c r="J60" t="n">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
       <c r="K60" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="L60" t="n">
         <v>0.5</v>
@@ -3100,19 +3100,19 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>61.3</v>
+        <v>66.5</v>
       </c>
       <c r="H61" t="n">
-        <v>14.4</v>
+        <v>15.1</v>
       </c>
       <c r="I61" t="n">
-        <v>7.4</v>
+        <v>8.1</v>
       </c>
       <c r="J61" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="K61" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="L61" t="n">
         <v>0.5</v>
@@ -3144,22 +3144,22 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>38.7</v>
+        <v>33.5</v>
       </c>
       <c r="H62" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
       <c r="I62" t="n">
-        <v>4.3</v>
+        <v>3.4</v>
       </c>
       <c r="J62" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="K62" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="L62" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="63">
@@ -3188,22 +3188,22 @@
         <v>100</v>
       </c>
       <c r="G63" t="n">
-        <v>36.4</v>
+        <v>35.7</v>
       </c>
       <c r="H63" t="n">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
       <c r="I63" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="K63" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L63" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -3232,22 +3232,22 @@
         <v>100</v>
       </c>
       <c r="G64" t="n">
-        <v>40.8</v>
+        <v>35.7</v>
       </c>
       <c r="H64" t="n">
-        <v>16.4</v>
+        <v>14.2</v>
       </c>
       <c r="I64" t="n">
-        <v>6.7</v>
+        <v>5.5</v>
       </c>
       <c r="J64" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="K64" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="L64" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="65">
@@ -3276,16 +3276,16 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>43.3</v>
+        <v>42.6</v>
       </c>
       <c r="H65" t="n">
-        <v>14.4</v>
+        <v>13.9</v>
       </c>
       <c r="I65" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="J65" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="K65" t="n">
         <v>0.3</v>
@@ -3320,7 +3320,7 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>19.1</v>
+        <v>18.8</v>
       </c>
       <c r="H66" t="n">
         <v>5.3</v>
@@ -3332,7 +3332,7 @@
         <v>0.2</v>
       </c>
       <c r="K66" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -3364,16 +3364,16 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>19.5</v>
+        <v>23.2</v>
       </c>
       <c r="H67" t="n">
-        <v>4</v>
+        <v>5.8</v>
       </c>
       <c r="I67" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
       <c r="J67" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3408,7 +3408,7 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
       <c r="H68" t="n">
         <v>1.1</v>
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="H69" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I69" t="n">
         <v>0.1</v>

</xml_diff>